<commit_message>
Experimental chapter specifications and justifications
</commit_message>
<xml_diff>
--- a/Corrections/Corrections Response.xlsx
+++ b/Corrections/Corrections Response.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\PhDThesis\Corrections\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFD04E42-C510-4D19-BF68-68F84964EC5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF3D0D4A-D1D8-40B2-B66F-75AA11CFB37B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{4546FF8B-BC23-429E-85B6-7F6A0D840A61}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{4546FF8B-BC23-429E-85B6-7F6A0D840A61}"/>
   </bookViews>
   <sheets>
     <sheet name="Tom Slatter + Amir Kadiric" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="153">
   <si>
     <t>Section</t>
   </si>
@@ -45,12 +45,6 @@
     <t>Correction</t>
   </si>
   <si>
-    <t>Validity</t>
-  </si>
-  <si>
-    <t>Intensity</t>
-  </si>
-  <si>
     <t>Abstract</t>
   </si>
   <si>
@@ -264,9 +258,6 @@
     <t>Accuracy of displacement measurements</t>
   </si>
   <si>
-    <t>Try locate data sheet. Comment on noise flaw, deviation at each frequency of B&amp;J and also laser vibrometer:</t>
-  </si>
-  <si>
     <t>How necessary is the iteration scheme here given the minimal impact of load on film? How does ignoring  this compare to other sources of error, for example accuracy of your location measurements? Add a short discussion with some values to illustrate  sensitivity of solution(s) to this if possible</t>
   </si>
   <si>
@@ -276,9 +267,6 @@
     <t>What acceleration is this from 0-15000rpm in 4s? Was this accounted for in the EHL film predictions? What entrainment speed? Are there inlet shear heating effects? You go through a lot of trouble to describe the 1D Reynolds solver but these other factors may be just as (or even more) important. Add brief discussion.</t>
   </si>
   <si>
-    <t>Quasistatic snapshots no considered in transient EHL. No inlet shear heating considered.</t>
-  </si>
-  <si>
     <t>Reference Hetzx approach in eq. 3.11</t>
   </si>
   <si>
@@ -405,9 +393,6 @@
     <t>No, justify. Find one area to put this justification.</t>
   </si>
   <si>
-    <t>Customer model</t>
-  </si>
-  <si>
     <t>Did not use Gupta corrections for this</t>
   </si>
   <si>
@@ -505,6 +490,12 @@
   </si>
   <si>
     <t>This is already explained in section 4.3.2, including what isn't modelled (flexible bodies in representative excitation model and stator tooth forces duer to minimal lateral contribution once resolved).</t>
+  </si>
+  <si>
+    <t>Light transmission fluid from industrial partner</t>
+  </si>
+  <si>
+    <t>Quasistatic snapshots not considered in transient EHL. No inlet shear heating considered at this stage. Will add comments regardin this later</t>
   </si>
 </sst>
 </file>
@@ -562,7 +553,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -585,6 +576,12 @@
         <fgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -600,7 +597,7 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -631,6 +628,10 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -968,18 +969,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57F42DE2-BF3F-4B4A-ACA4-1B57B73DE292}">
-  <dimension ref="A1:F94"/>
+  <dimension ref="A1:D94"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34.7109375" customWidth="1"/>
     <col min="2" max="2" width="80" customWidth="1"/>
     <col min="3" max="3" width="69" customWidth="1"/>
     <col min="4" max="4" width="42.28515625" customWidth="1"/>
-    <col min="5" max="5" width="11.5703125" customWidth="1"/>
-    <col min="6" max="6" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -987,1397 +986,872 @@
         <v>1</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E1" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="B2" s="3" t="s">
         <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>5</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="6"/>
-      <c r="E2" s="2">
-        <v>5</v>
-      </c>
-      <c r="F2" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4"/>
       <c r="B3" s="6" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="6"/>
-      <c r="E3" s="2">
-        <v>5</v>
-      </c>
-      <c r="F3" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="3"/>
-      <c r="E4" s="2">
+    </row>
+    <row r="5" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
-        <v>6</v>
-      </c>
       <c r="B5" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="D5" s="1"/>
-      <c r="E5" s="2">
-        <v>4</v>
-      </c>
-      <c r="F5" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4"/>
       <c r="B6" s="7" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C6" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="D6" s="1"/>
+    </row>
+    <row r="7" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="D6" s="1"/>
-      <c r="E6" s="2">
-        <v>4</v>
-      </c>
-      <c r="F6" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>132</v>
-      </c>
       <c r="D7" s="1"/>
-      <c r="E7" s="2">
-        <v>3</v>
-      </c>
-      <c r="F7" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4"/>
       <c r="B8" s="7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="D8" s="1"/>
-      <c r="E8" s="2">
-        <v>2</v>
-      </c>
-      <c r="F8" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4"/>
       <c r="B9" s="7" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="D9" s="1"/>
-      <c r="E9" s="2">
-        <v>1</v>
-      </c>
-      <c r="F9" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4"/>
       <c r="B10" s="7" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="D10" s="1"/>
-      <c r="E10" s="2">
-        <v>5</v>
-      </c>
-      <c r="F10" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4"/>
       <c r="B11" s="7" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="E11" s="2">
-        <v>3</v>
-      </c>
-      <c r="F11" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4"/>
       <c r="B12" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C12" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="C12" s="9" t="s">
-        <v>41</v>
-      </c>
       <c r="D12" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="E12" s="2">
-        <v>1</v>
-      </c>
-      <c r="F12" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="4"/>
       <c r="B13" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="D13" s="1"/>
-      <c r="E13" s="2">
-        <v>4</v>
-      </c>
-      <c r="F13" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="4"/>
       <c r="B14" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="D14" s="1"/>
-      <c r="E14" s="2">
-        <v>3</v>
-      </c>
-      <c r="F14" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="4"/>
       <c r="B15" s="7" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="E15" s="2">
-        <v>2</v>
-      </c>
-      <c r="F15" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4"/>
       <c r="B16" s="7" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="E16" s="2">
-        <v>2</v>
-      </c>
-      <c r="F16" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="4"/>
       <c r="B17" s="7" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="E17" s="2">
-        <v>2</v>
-      </c>
-      <c r="F17" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="4"/>
       <c r="B18" s="7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="D18" s="1"/>
-      <c r="E18" s="2">
-        <v>5</v>
-      </c>
-      <c r="F18" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:4" ht="75" x14ac:dyDescent="0.25">
       <c r="A19" s="4"/>
       <c r="B19" s="7" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E19" s="2">
-        <v>3</v>
-      </c>
-      <c r="F19" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4"/>
       <c r="B20" s="7" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="D20" s="1"/>
-      <c r="E20" s="2">
-        <v>4</v>
-      </c>
-      <c r="F20" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="4"/>
       <c r="B21" s="7" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="D21" s="1"/>
-      <c r="E21" s="2">
-        <v>1</v>
-      </c>
-      <c r="F21" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="4"/>
       <c r="B22" s="7" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="D22" s="1"/>
-      <c r="E22" s="2">
-        <v>4</v>
-      </c>
-      <c r="F22" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="4"/>
       <c r="B23" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="D23" s="1"/>
-      <c r="E23" s="2">
-        <v>4</v>
-      </c>
-      <c r="F23" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="24" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="4"/>
       <c r="B24" s="7" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="D24" s="1"/>
-      <c r="E24" s="2">
-        <v>4</v>
-      </c>
-      <c r="F24" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="4"/>
       <c r="B25" s="7" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="D25" s="1"/>
-      <c r="E25" s="2">
-        <v>1</v>
-      </c>
-      <c r="F25" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="4"/>
       <c r="B26" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="E26" s="2">
-        <v>4</v>
-      </c>
-      <c r="F26" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="4"/>
       <c r="B27" s="7" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="E27" s="2">
-        <v>3</v>
-      </c>
-      <c r="F27" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="4"/>
       <c r="B28" s="7" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="D28" s="1"/>
-      <c r="E28" s="2">
-        <v>2</v>
-      </c>
-      <c r="F28" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="4"/>
       <c r="B29" s="7" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="D29" s="1"/>
-      <c r="E29" s="2">
-        <v>4</v>
-      </c>
-      <c r="F29" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="30" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="4"/>
       <c r="B30" s="7" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="D30" s="1"/>
-      <c r="E30" s="2">
-        <v>4</v>
-      </c>
-      <c r="F30" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="31" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="4"/>
       <c r="B31" s="7" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="E31" s="2">
-        <v>3</v>
-      </c>
-      <c r="F31" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="4"/>
       <c r="B32" s="7" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="D32" s="1"/>
-      <c r="E32" s="2">
-        <v>4</v>
-      </c>
-      <c r="F32" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="33" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="4"/>
       <c r="B33" s="7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C33" s="9" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="D33" s="1"/>
-      <c r="E33" s="2">
-        <v>4</v>
-      </c>
-      <c r="F33" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="34" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="4"/>
       <c r="B34" s="7" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" s="1"/>
-      <c r="E34" s="2">
-        <v>4</v>
-      </c>
-      <c r="F34" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="35" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="4"/>
       <c r="B35" s="7" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="1"/>
-      <c r="E35" s="2">
-        <v>4</v>
-      </c>
-      <c r="F35" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="36" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="4"/>
       <c r="B36" s="7" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="D36" s="1"/>
-      <c r="E36" s="2">
-        <v>2</v>
-      </c>
-      <c r="F36" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="37" spans="1:4" ht="90" x14ac:dyDescent="0.25">
       <c r="A37" s="4"/>
       <c r="B37" s="7" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" s="1"/>
-      <c r="E37" s="2">
-        <v>5</v>
-      </c>
-      <c r="F37" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="38" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B38" s="7"/>
       <c r="C38" s="2"/>
       <c r="D38" s="1"/>
-      <c r="E38" s="2"/>
-      <c r="F38" s="2"/>
-    </row>
-    <row r="39" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="39" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="4"/>
       <c r="B39" s="7" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="D39" s="1"/>
-      <c r="E39" s="2">
-        <v>2</v>
-      </c>
-      <c r="F39" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="40" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="4"/>
       <c r="B40" s="7" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="D40" s="1"/>
-      <c r="E40" s="2">
-        <v>2</v>
-      </c>
-      <c r="F40" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="41" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="4"/>
       <c r="B41" s="7" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" s="1"/>
-      <c r="E41" s="2">
-        <v>4</v>
-      </c>
-      <c r="F41" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="42" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="4"/>
       <c r="B42" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="C42" s="2"/>
-      <c r="D42" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="E42" s="2">
-        <v>4</v>
-      </c>
-      <c r="F42" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C42" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="D42" s="1"/>
+    </row>
+    <row r="43" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A43" s="4"/>
       <c r="B43" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="C43" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="D43" s="1"/>
-      <c r="E43" s="2">
-        <v>4</v>
-      </c>
-      <c r="F43" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+        <v>75</v>
+      </c>
+      <c r="C43" s="2"/>
+      <c r="D43" s="1" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="4"/>
       <c r="B44" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C44" s="2"/>
+        <v>76</v>
+      </c>
+      <c r="C44" s="8" t="s">
+        <v>137</v>
+      </c>
       <c r="D44" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="E44" s="2">
-        <v>3</v>
-      </c>
-      <c r="F44" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="4"/>
       <c r="B45" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="C45" s="8" t="s">
-        <v>142</v>
+        <v>77</v>
+      </c>
+      <c r="C45" s="9" t="s">
+        <v>138</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="E45" s="2">
-        <v>4</v>
-      </c>
-      <c r="F45" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="4"/>
       <c r="B46" s="7" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C46" s="9" t="s">
-        <v>143</v>
+        <v>125</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="E46" s="2">
-        <v>4</v>
-      </c>
-      <c r="F46" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="4"/>
       <c r="B47" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="C47" s="9" t="s">
-        <v>130</v>
-      </c>
+        <v>79</v>
+      </c>
+      <c r="C47" s="2"/>
       <c r="D47" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="E47" s="2">
-        <v>3</v>
-      </c>
-      <c r="F47" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="4"/>
       <c r="B48" s="7" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="E48" s="2">
-        <v>3</v>
-      </c>
-      <c r="F48" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A49" s="4"/>
       <c r="B49" s="7" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="E49" s="2">
-        <v>3</v>
-      </c>
-      <c r="F49" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="4"/>
       <c r="B50" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="C50" s="2"/>
-      <c r="D50" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="E50" s="2">
-        <v>3</v>
-      </c>
-      <c r="F50" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>84</v>
+      </c>
+      <c r="C50" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="D50" s="1"/>
+    </row>
+    <row r="51" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="4"/>
       <c r="B51" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="C51" s="8" t="s">
-        <v>144</v>
+        <v>85</v>
+      </c>
+      <c r="C51" s="9" t="s">
+        <v>147</v>
       </c>
       <c r="D51" s="1"/>
-      <c r="E51" s="2">
-        <v>4</v>
-      </c>
-      <c r="F51" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="52" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="4"/>
       <c r="B52" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="C52" s="9" t="s">
-        <v>152</v>
+        <v>86</v>
+      </c>
+      <c r="C52" s="8" t="s">
+        <v>146</v>
       </c>
       <c r="D52" s="1"/>
-      <c r="E52" s="2">
-        <v>3</v>
-      </c>
-      <c r="F52" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="53" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="4"/>
       <c r="B53" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="C53" s="8" t="s">
-        <v>151</v>
+        <v>87</v>
+      </c>
+      <c r="C53" s="9" t="s">
+        <v>140</v>
       </c>
       <c r="D53" s="1"/>
-      <c r="E53" s="2">
-        <v>3</v>
-      </c>
-      <c r="F53" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="4"/>
-      <c r="B54" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="C54" s="9" t="s">
-        <v>145</v>
-      </c>
+    </row>
+    <row r="54" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="11"/>
+      <c r="B54" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C54" s="2"/>
       <c r="D54" s="1"/>
-      <c r="E54" s="2">
-        <v>4</v>
-      </c>
-      <c r="F54" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="55" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="12"/>
       <c r="B55" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" s="1"/>
-      <c r="E55" s="2">
-        <v>3</v>
-      </c>
-      <c r="F55" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="4"/>
+    </row>
+    <row r="56" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="12"/>
       <c r="B56" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" s="1"/>
-      <c r="E56" s="2">
-        <v>4</v>
-      </c>
-      <c r="F56" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="4"/>
+    </row>
+    <row r="57" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="12"/>
       <c r="B57" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" s="1"/>
-      <c r="E57" s="2">
-        <v>3</v>
-      </c>
-      <c r="F57" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="4"/>
-      <c r="B58" s="1" t="s">
-        <v>18</v>
+    </row>
+    <row r="58" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="12"/>
+      <c r="B58" s="7" t="s">
+        <v>72</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" s="1"/>
-      <c r="E58" s="2">
-        <v>3</v>
-      </c>
-      <c r="F58" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="59" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="4"/>
       <c r="B59" s="7" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" s="1"/>
-      <c r="E59" s="2">
-        <v>3</v>
-      </c>
-      <c r="F59" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="60" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="4"/>
       <c r="B60" s="7" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" s="1"/>
-      <c r="E60" s="2">
-        <v>3</v>
-      </c>
-      <c r="F60" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="61" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" s="1"/>
-      <c r="E61" s="2">
-        <v>3</v>
-      </c>
-      <c r="F61" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="62" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="4"/>
       <c r="B62" s="7" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" s="1"/>
-      <c r="E62" s="2">
-        <v>3</v>
-      </c>
-      <c r="F62" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="63" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="4"/>
       <c r="B63" s="7" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C63" s="9" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="D63" s="1"/>
-      <c r="E63" s="2">
-        <v>3</v>
-      </c>
-      <c r="F63" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="64" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="4"/>
       <c r="B64" s="7" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" s="1"/>
-      <c r="E64" s="2">
-        <v>3</v>
-      </c>
-      <c r="F64" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="65" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="4"/>
       <c r="B65" s="7" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="C65" s="8" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="D65" s="1"/>
-      <c r="E65" s="2">
-        <v>3</v>
-      </c>
-      <c r="F65" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="66" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="4"/>
       <c r="B66" s="7" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="C66" s="2"/>
       <c r="D66" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="E66" s="2">
-        <v>3</v>
-      </c>
-      <c r="F66" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="4"/>
       <c r="B67" s="7" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="C67" s="2"/>
       <c r="D67" s="1"/>
-      <c r="E67" s="2">
-        <v>3</v>
-      </c>
-      <c r="F67" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="68" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="4"/>
       <c r="B68" s="7" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="C68" s="2"/>
       <c r="D68" s="1"/>
-      <c r="E68" s="2">
-        <v>2</v>
-      </c>
-      <c r="F68" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="69" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="4"/>
       <c r="B69" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C69" s="8" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="D69" s="1"/>
-      <c r="E69" s="2">
-        <v>2</v>
-      </c>
-      <c r="F69" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="70" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="4"/>
       <c r="B70" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C70" s="2"/>
       <c r="D70" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="E70" s="2">
-        <v>2</v>
-      </c>
-      <c r="F70" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="4"/>
       <c r="B71" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C71" s="9" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="D71" s="1"/>
-      <c r="E71" s="2">
-        <v>4</v>
-      </c>
-      <c r="F71" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="72" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="4"/>
       <c r="B72" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C72" s="2"/>
       <c r="D72" s="1"/>
-      <c r="E72" s="2">
-        <v>4</v>
-      </c>
-      <c r="F72" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="73" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="4"/>
       <c r="B73" s="7" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="C73" s="2"/>
       <c r="D73" s="1"/>
-      <c r="E73" s="2">
-        <v>4</v>
-      </c>
-      <c r="F73" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="74" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C74" s="2"/>
       <c r="D74" s="1"/>
-      <c r="E74" s="2">
-        <v>4</v>
-      </c>
-      <c r="F74" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" ht="75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="75" spans="1:4" ht="75" x14ac:dyDescent="0.25">
       <c r="A75" s="4"/>
       <c r="B75" s="7" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="C75" s="2"/>
       <c r="D75" s="1"/>
-      <c r="E75" s="2">
-        <v>3</v>
-      </c>
-      <c r="F75" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="76" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="76" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="4"/>
       <c r="B76" s="7" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="C76" s="2"/>
       <c r="D76" s="1"/>
-      <c r="E76" s="2">
-        <v>3</v>
-      </c>
-      <c r="F76" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="77" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="77" spans="1:4" ht="69" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="4"/>
       <c r="B77" s="7" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="C77" s="2"/>
       <c r="D77" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="E77" s="2">
-        <v>4</v>
-      </c>
-      <c r="F77" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="78" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="4"/>
       <c r="B78" s="7" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="C78" s="2"/>
       <c r="D78" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="E78" s="2">
-        <v>4</v>
-      </c>
-      <c r="F78" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="4"/>
       <c r="B79" s="7" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C79" s="9" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E79" s="2">
-        <v>1</v>
-      </c>
-      <c r="F79" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="80" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="4"/>
       <c r="B80" s="7" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="C80" s="8" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E80" s="2">
-        <v>1</v>
-      </c>
-      <c r="F80" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="81" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="4"/>
       <c r="B81" s="7" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C81" s="2"/>
       <c r="D81" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="E81" s="2">
-        <v>3</v>
-      </c>
-      <c r="F81" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="82" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="4"/>
       <c r="B82" s="7" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="C82" s="2"/>
       <c r="D82" s="1"/>
-      <c r="E82" s="2">
-        <v>4</v>
-      </c>
-      <c r="F82" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="83" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="83" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="4"/>
       <c r="B83" s="7" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C83" s="2"/>
       <c r="D83" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="E83" s="2">
-        <v>3</v>
-      </c>
-      <c r="F83" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="84" spans="1:6" ht="105" x14ac:dyDescent="0.25">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" ht="105" x14ac:dyDescent="0.25">
       <c r="A84" s="4"/>
       <c r="B84" s="7" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="C84" s="2"/>
       <c r="D84" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="E84" s="2">
-        <v>3</v>
-      </c>
-      <c r="F84" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="85" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A85" s="4"/>
       <c r="B85" s="7" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C85" s="2"/>
       <c r="D85" s="1"/>
-      <c r="E85" s="2">
-        <v>3</v>
-      </c>
-      <c r="F85" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="86" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="86" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C86" s="2"/>
       <c r="D86" s="1"/>
-      <c r="E86" s="2">
-        <v>5</v>
-      </c>
-      <c r="F86" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="87" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="4"/>
       <c r="B87" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C87" s="2"/>
       <c r="D87" s="1"/>
-      <c r="E87" s="2">
-        <v>5</v>
-      </c>
-      <c r="F87" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="88" spans="1:6" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="88" spans="1:4" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="4"/>
       <c r="B88" s="7" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C88" s="9" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="D88" s="1"/>
-      <c r="E88" s="2">
-        <v>3</v>
-      </c>
-      <c r="F88" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="89" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="89" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A89" s="4"/>
       <c r="B89" s="1"/>
       <c r="D89" s="1"/>
     </row>
-    <row r="90" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A90" s="4"/>
     </row>
-    <row r="91" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A91" s="4"/>
     </row>
-    <row r="92" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A92" s="4"/>
     </row>
-    <row r="93" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A93" s="4"/>
     </row>
-    <row r="94" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A94" s="4"/>
     </row>
   </sheetData>
@@ -2395,12 +1869,12 @@
   <sheetData>
     <row r="2" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
     </row>
     <row r="3" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>